<commit_message>
Remove leftover waveform graphs
</commit_message>
<xml_diff>
--- a/MUSCRadOncIGRT.xlsx
+++ b/MUSCRadOncIGRT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr saveExternalLinkValues="0" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\workspace\EquipTestingSpreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA1080A-6185-43DC-9F34-0BA82AAABF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF7055A-CDDF-4387-9B9D-E1AA272CAD69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gen_form" sheetId="1" r:id="rId1"/>
@@ -7416,47 +7416,8 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="22" fillId="6" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="22" fillId="6" borderId="94" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="22" fillId="6" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="22" fillId="6" borderId="118" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="8" fillId="0" borderId="116" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7482,11 +7443,50 @@
     <xf numFmtId="10" fontId="8" fillId="0" borderId="125" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="22" fillId="6" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="22" fillId="6" borderId="94" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="22" fillId="6" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="22" fillId="6" borderId="118" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -7532,11 +7532,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C6500"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7547,16 +7547,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7582,6 +7572,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -7592,21 +7592,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C6500"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7670,11 +7670,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7690,11 +7690,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10735,1361 +10735,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>68</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B4E2258-7149-0D4A-DC78-2DC267A7C5E6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="8801100"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>69</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>93</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAC5E0A4-4532-A77F-754A-AF25CC9B8404}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="13801725"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>94</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>118</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C84703FF-755D-4D78-1A1A-2634D8B7053B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="18802350"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>119</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>143</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 8">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12807CDC-3733-155E-FA53-B0CA92BF993B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="23802975"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>144</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>168</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 10">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5B46BED-BB19-A38F-5689-19C9A1F7A6AB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="28803600"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>169</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>193</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Picture 12">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87D338A2-B8C7-404B-3ABF-96BEBB54F23C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="33804225"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>194</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>218</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Picture 14">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D390C269-3C0B-7543-21D3-0EB5FD3EAD1F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="38804850"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>219</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>243</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Picture 16">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BDA3F9D-FD70-09FD-0C8D-92BF273F4F7F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="43805475"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>244</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>268</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Picture 18">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D383A18-D0C0-EF6A-1F7D-EB2C12A1FA0C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="48806100"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>269</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>293</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="Picture 20">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13C336EC-5A4D-3344-186D-F905DE18A9C4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="53806725"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>294</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>318</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Picture 22">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20B51CFE-2FC9-DF26-B62A-4E423AA8D503}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="58807350"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>319</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>343</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Picture 24">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA8821CE-4BB5-DF41-11EA-27D937392BF8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="63807975"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>344</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>368</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="Picture 26">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{42811A83-6D38-6F3F-1535-BCBDB55F0201}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="68808600"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>369</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>393</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="29" name="Picture 28">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47524E8C-AB1C-FFE3-A731-047BEF3C337B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="73809225"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>394</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>418</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="31" name="Picture 30">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{275477AD-5282-D895-7AA4-9B7729B94D00}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="78809850"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>419</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>443</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="33" name="Picture 32">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E371589-636B-CD13-347E-7222E43D27BE}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="83810475"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>444</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>468</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="35" name="Picture 34">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{41B8C381-CEC9-D3F9-51FB-EE28D51C6225}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="88811100"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>469</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>493</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="37" name="Picture 36">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5AC0C3C6-EE90-21A5-B56A-1FB60AFCC1F4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="93811725"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>494</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>518</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="39" name="Picture 38">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9511D79-97DE-5D1B-1860-4579DFE5E01A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="98812350"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>519</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>543</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="41" name="Picture 40">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF05DC21-E93A-1F3C-F442-A40E2FD9C61D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="103812975"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>544</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>568</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="43" name="Picture 42">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CB91488-6094-4642-B755-8449DE3D617A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="108813600"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>569</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>593</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="45" name="Picture 44">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2518977-AA8D-5C7A-2233-EE3EA5ADCF1D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="113814225"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>594</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>618</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="47" name="Picture 46">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03027312-1D53-7FF1-0E72-2134484EB2B8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="118814850"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>619</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>643</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="49" name="Picture 48">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DBD8CCC-23C6-167D-B497-C7C233D8AEB3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="123815475"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>644</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>668</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="51" name="Picture 50">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52BBD2C5-EE27-8EC5-B6B2-AD4AEEC631E2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="128816100"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>669</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>693</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="53" name="Picture 52">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5276440A-6D58-011B-EFEA-433B4FC6E414}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="133816725"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>694</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>718</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="55" name="Picture 54">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45D65A35-1020-9638-86DF-8391475B0998}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="138817350"/>
-          <a:ext cx="7143750" cy="4981575"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -15991,10 +14636,10 @@
       <c r="L67" s="465" t="s">
         <v>265</v>
       </c>
-      <c r="U67" s="840" t="s">
+      <c r="U67" s="849" t="s">
         <v>192</v>
       </c>
-      <c r="V67" s="841"/>
+      <c r="V67" s="850"/>
       <c r="X67" s="455" t="s">
         <v>265</v>
       </c>
@@ -16107,10 +14752,10 @@
       <c r="F71" s="87" t="s">
         <v>293</v>
       </c>
-      <c r="J71" s="838" t="s">
+      <c r="J71" s="847" t="s">
         <v>269</v>
       </c>
-      <c r="K71" s="839"/>
+      <c r="K71" s="848"/>
       <c r="L71" s="465" t="s">
         <v>265</v>
       </c>
@@ -19025,11 +17670,11 @@
       <c r="AE126" s="330" t="s">
         <v>449</v>
       </c>
-      <c r="AH126" s="854" t="str">
+      <c r="AH126" s="841" t="str">
         <f>ROUND(I605,1)&amp;" kV"</f>
         <v>80 kV</v>
       </c>
-      <c r="AI126" s="854"/>
+      <c r="AI126" s="841"/>
     </row>
     <row r="127" spans="1:35" ht="11.25" customHeight="1" thickBot="1">
       <c r="A127" s="418">
@@ -21803,22 +20448,22 @@
         <v>265</v>
       </c>
       <c r="M186" s="110"/>
-      <c r="O186" s="850" t="s">
+      <c r="O186" s="859" t="s">
         <v>367</v>
       </c>
-      <c r="P186" s="851"/>
-      <c r="Q186" s="850" t="s">
+      <c r="P186" s="860"/>
+      <c r="Q186" s="859" t="s">
         <v>368</v>
       </c>
-      <c r="R186" s="851"/>
-      <c r="S186" s="844" t="s">
+      <c r="R186" s="860"/>
+      <c r="S186" s="853" t="s">
         <v>369</v>
       </c>
-      <c r="T186" s="845"/>
-      <c r="U186" s="842" t="s">
+      <c r="T186" s="854"/>
+      <c r="U186" s="851" t="s">
         <v>373</v>
       </c>
-      <c r="V186" s="843"/>
+      <c r="V186" s="852"/>
       <c r="W186" s="59"/>
       <c r="X186" s="455" t="s">
         <v>265</v>
@@ -21843,28 +20488,28 @@
       <c r="L187" s="465" t="s">
         <v>265</v>
       </c>
-      <c r="M187" s="848" t="s">
+      <c r="M187" s="857" t="s">
         <v>374</v>
       </c>
-      <c r="N187" s="849"/>
-      <c r="O187" s="844" t="str">
+      <c r="N187" s="858"/>
+      <c r="O187" s="853" t="str">
         <f>"("&amp;TBCM_IN&amp;")"</f>
         <v>(cm)</v>
       </c>
-      <c r="P187" s="845"/>
-      <c r="Q187" s="844" t="str">
+      <c r="P187" s="854"/>
+      <c r="Q187" s="853" t="str">
         <f>"("&amp;TBCM_IN&amp;")"</f>
         <v>(cm)</v>
       </c>
-      <c r="R187" s="845"/>
-      <c r="S187" s="846" t="s">
+      <c r="R187" s="854"/>
+      <c r="S187" s="855" t="s">
         <v>370</v>
       </c>
-      <c r="T187" s="847"/>
-      <c r="U187" s="844" t="s">
+      <c r="T187" s="856"/>
+      <c r="U187" s="853" t="s">
         <v>369</v>
       </c>
-      <c r="V187" s="845"/>
+      <c r="V187" s="854"/>
       <c r="W187" s="59"/>
       <c r="X187" s="455" t="s">
         <v>265</v>
@@ -28492,10 +27137,10 @@
         <v>369</v>
       </c>
       <c r="G311" s="563"/>
-      <c r="H311" s="855" t="s">
+      <c r="H311" s="842" t="s">
         <v>373</v>
       </c>
-      <c r="I311" s="856"/>
+      <c r="I311" s="843"/>
       <c r="J311" s="327"/>
       <c r="K311" s="59"/>
       <c r="L311" s="465" t="s">
@@ -39589,7 +38234,7 @@
         <f>IF(OR(H540="",AND(LFMAS="",SFMAS=""),AND($C$539="mA",D540="")),"",IF($C$539="mAs",H540/C540,H540/(C540*D540)))</f>
         <v/>
       </c>
-      <c r="J540" s="852" t="str">
+      <c r="J540" s="839" t="str">
         <f>IF(OR(I540="",I541=""),"",(MAX(I540:I541)-MIN(I540:I541))/(MAX(I540:I541)+MIN(I540:I541)))</f>
         <v/>
       </c>
@@ -39647,7 +38292,7 @@
         <f>IF(OR(H541="",AND(LFMAS="",SFMAS=""),AND($C$539="mA",D541="")),"",IF($C$539="mAs",H541/C541,H541/(C541*D541)))</f>
         <v/>
       </c>
-      <c r="J541" s="853"/>
+      <c r="J541" s="840"/>
       <c r="K541" s="216" t="str">
         <f>IF(J540="","TBD",IF(J540&gt;0.1,"NO","YES"))</f>
         <v>TBD</v>
@@ -39715,7 +38360,7 @@
         <f>IF(OR(H542="",AND(LFMAS="",SFMAS=""),AND($C$539="mA",D542="")),"",IF($C$539="mAs",H542/C542,H542/(C542*D542)))</f>
         <v/>
       </c>
-      <c r="J542" s="852" t="str">
+      <c r="J542" s="839" t="str">
         <f>IF(OR(I540="",I542=""),"",(MAX(I540:I544)-MIN(I540:I544))/(MAX(I540:I544)+MIN(I540:I544)))</f>
         <v/>
       </c>
@@ -39786,7 +38431,7 @@
         <f>IF(OR(H543="",AND(LFMAS="",SFMAS=""),AND($C$539="mA",D543="")),"",IF($C$539="mAs",H543/C543,H543/(C543*D543)))</f>
         <v/>
       </c>
-      <c r="J543" s="859"/>
+      <c r="J543" s="846"/>
       <c r="K543" s="215" t="s">
         <v>108</v>
       </c>
@@ -39856,7 +38501,7 @@
         <f>IF(OR(H544="",AND(LFMAS="",SFMAS=""),AND($C$539="mA",D544="")),"",IF($C$539="mAs",H544/C544,H544/(C544*D544)))</f>
         <v/>
       </c>
-      <c r="J544" s="853"/>
+      <c r="J544" s="840"/>
       <c r="K544" s="216" t="str">
         <f>IF(J542="","TBD",IF(J542&gt;0.1,"NO","YES"))</f>
         <v>TBD</v>
@@ -40422,7 +39067,7 @@
         <f>IF(OR(H555="",AND(LFMAS="",SFMAS=""),AND($C$554="mA",D555="")),"",IF($C$554="mAs",H555/C555,H555/(C555*D555)))</f>
         <v/>
       </c>
-      <c r="J555" s="852" t="str">
+      <c r="J555" s="839" t="str">
         <f>IF(OR(I555="",I556=""),"",(MAX(I555:I556)-MIN(I555:I556))/(MAX(I555:I556)+MIN(I555:I556)))</f>
         <v/>
       </c>
@@ -40495,7 +39140,7 @@
         <f>IF(OR(H556="",AND(LFMAS="",SFMAS=""),AND($C$554="mA",D556="")),"",IF($C$554="mAs",H556/C556,H556/(C556*D556)))</f>
         <v/>
       </c>
-      <c r="J556" s="853"/>
+      <c r="J556" s="840"/>
       <c r="K556" s="216" t="str">
         <f>IF(J555="","TBD",IF(J555&gt;0.1,"NO","YES"))</f>
         <v>TBD</v>
@@ -40562,7 +39207,7 @@
         <f>IF(OR(H557="",AND(LFMAS="",SFMAS=""),AND($C$554="mA",D557="")),"",IF($C$554="mAs",H557/C557,H557/(C557*D557)))</f>
         <v/>
       </c>
-      <c r="J557" s="852" t="str">
+      <c r="J557" s="839" t="str">
         <f>IF(OR(I555="",I557=""),"",(MAX(I555:I559)-MIN(I555:I559))/(MAX(I555:I559)+MIN(I555:I559)))</f>
         <v/>
       </c>
@@ -40629,7 +39274,7 @@
         <f>IF(OR(H558="",AND(LFMAS="",SFMAS=""),AND($C$554="mA",D558="")),"",IF($C$554="mAs",H558/C558,H558/(C558*D558)))</f>
         <v/>
       </c>
-      <c r="J558" s="859"/>
+      <c r="J558" s="846"/>
       <c r="K558" s="215" t="s">
         <v>108</v>
       </c>
@@ -40695,7 +39340,7 @@
         <f>IF(OR(H559="",AND(LFMAS="",SFMAS=""),AND($C$554="mA",D559="")),"",IF($C$554="mAs",H559/C559,H559/(C559*D559)))</f>
         <v/>
       </c>
-      <c r="J559" s="853"/>
+      <c r="J559" s="840"/>
       <c r="K559" s="216" t="str">
         <f>IF(J557="","TBD",IF(J557&gt;0.1,"NO","YES"))</f>
         <v>TBD</v>
@@ -42841,8 +41486,8 @@
         <v>32</v>
       </c>
       <c r="B626" s="54"/>
-      <c r="E626" s="857"/>
-      <c r="F626" s="857"/>
+      <c r="E626" s="844"/>
+      <c r="F626" s="844"/>
       <c r="I626" s="37"/>
       <c r="K626" s="59"/>
       <c r="L626" s="465" t="s">
@@ -42859,8 +41504,8 @@
       <c r="B627" s="54"/>
       <c r="C627" s="37"/>
       <c r="D627" s="37"/>
-      <c r="E627" s="858"/>
-      <c r="F627" s="857"/>
+      <c r="E627" s="845"/>
+      <c r="F627" s="844"/>
       <c r="H627" s="42"/>
       <c r="I627" s="37"/>
       <c r="K627" s="59"/>
@@ -46519,14 +45164,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="19">
-    <mergeCell ref="J540:J541"/>
-    <mergeCell ref="AH126:AI126"/>
-    <mergeCell ref="H311:I311"/>
-    <mergeCell ref="E626:E627"/>
-    <mergeCell ref="F626:F627"/>
-    <mergeCell ref="J542:J544"/>
-    <mergeCell ref="J555:J556"/>
-    <mergeCell ref="J557:J559"/>
     <mergeCell ref="J71:K71"/>
     <mergeCell ref="U67:V67"/>
     <mergeCell ref="U186:V186"/>
@@ -46538,6 +45175,14 @@
     <mergeCell ref="O186:P186"/>
     <mergeCell ref="Q186:R186"/>
     <mergeCell ref="S186:T186"/>
+    <mergeCell ref="J540:J541"/>
+    <mergeCell ref="AH126:AI126"/>
+    <mergeCell ref="H311:I311"/>
+    <mergeCell ref="E626:E627"/>
+    <mergeCell ref="F626:F627"/>
+    <mergeCell ref="J542:J544"/>
+    <mergeCell ref="J555:J556"/>
+    <mergeCell ref="J557:J559"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <conditionalFormatting sqref="B779">
@@ -46660,15 +45305,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q494:S494 Q509:S509">
-    <cfRule type="cellIs" dxfId="20" priority="41" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="43" operator="between">
       <formula>-0.25</formula>
+      <formula>0.25</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="19" priority="42" operator="greaterThan">
       <formula>0.25</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="43" operator="between">
+    <cfRule type="cellIs" dxfId="18" priority="41" operator="lessThan">
       <formula>-0.25</formula>
-      <formula>0.25</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q494:S494 V494 Q509:S509 V509">
@@ -46702,33 +45347,33 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U189:V190">
-    <cfRule type="cellIs" dxfId="11" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="48" operator="equal">
+      <formula>"NA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="47" operator="equal">
       <formula>"NO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="48" operator="equal">
-      <formula>"NA"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="9" priority="49" operator="equal">
       <formula>"YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U354:W363">
-    <cfRule type="cellIs" dxfId="8" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="40" operator="equal">
+      <formula>"NO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="39" operator="equal">
       <formula>"YES"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="40" operator="equal">
-      <formula>"NO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V244 V261 U294:W294 V314:W314 V395 V398 V411 V413 V421 S472:S473 V494 V509">
-    <cfRule type="cellIs" dxfId="6" priority="44" operator="equal">
-      <formula>"TBD"</formula>
+    <cfRule type="cellIs" dxfId="6" priority="46" operator="equal">
+      <formula>"NO"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="5" priority="45" operator="equal">
       <formula>"YES"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="46" operator="equal">
-      <formula>"NO"</formula>
+    <cfRule type="cellIs" dxfId="4" priority="44" operator="equal">
+      <formula>"TBD"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V352">
@@ -46802,10 +45447,10 @@
   <sheetFormatPr defaultRowHeight="15.6"/>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="860" t="s">
+      <c r="A1" s="861" t="s">
         <v>523</v>
       </c>
-      <c r="B1" s="860"/>
+      <c r="B1" s="861"/>
       <c r="D1" s="3"/>
       <c r="E1" s="312" t="s">
         <v>3</v>
@@ -47290,7 +45935,7 @@
       <c r="A29" s="723" t="s">
         <v>833</v>
       </c>
-      <c r="B29" s="861" t="s">
+      <c r="B29" s="838" t="s">
         <v>834</v>
       </c>
     </row>
@@ -47298,7 +45943,7 @@
       <c r="A30" s="723" t="s">
         <v>835</v>
       </c>
-      <c r="B30" s="861" t="s">
+      <c r="B30" s="838" t="s">
         <v>836</v>
       </c>
     </row>
@@ -48364,7 +47009,6 @@
     </customSheetView>
   </customSheetViews>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>